<commit_message>
feat(manifest): implement Manifest Validation contract (ELK-ORCA-PROD-004)
- Enhance scripts/validate-manifest.js with CLI args, event/artifact emission,
  and proper exit codes
- Emit orca.manifest_validated event and app.manifest artifact on success
- Emit orca.manifest_validation_failed event on failure
- Add 4 synthetic manifest fixtures (valid + 3 negative cases)
- Add tests/unit/manifest-validation.test.js with 7 tests
- Fix EventBus _persistEvent to preserve source and correlationId
- Document operator behavior in docs/notes/MANIFEST_VALIDATION_OPERATOR.md
- Update roadmap CSV/XLSX: ELK-ORCA-PROD-004 marked Done

Verification: npm run manifest && node --test tests/unit/manifest-validation.test.js
</commit_message>
<xml_diff>
--- a/docs/plans/2026-06-15_ELKHEDR_ORCA_APP_PRODUCTION_ROADMAP.xlsx
+++ b/docs/plans/2026-06-15_ELKHEDR_ORCA_APP_PRODUCTION_ROADMAP.xlsx
@@ -992,7 +992,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Proposed</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -1057,12 +1057,12 @@
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>cd elkhedr-orca &amp;&amp; npm run manifest</t>
+          <t>cd elkhedr-orca &amp;&amp; npm run manifest &amp;&amp; node --test tests/unit/manifest-validation.test.js</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>Pending implementation.</t>
+          <t>Enhanced scripts/validate-manifest.js to validate arbitrary manifest paths, emit orca.manifest_validated event, write app.manifest artifact, and emit orca.manifest_validation_failed on failure. Added 4 synthetic fixtures and 7 unit tests. Operator docs at docs/notes/MANIFEST_VALIDATION_OPERATOR.md.</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">

</xml_diff>